<commit_message>
Approve six Universal Adept abilities
Adds The Strong Arm, The Last Word, The Impossible Escape, A Name Worth Knowing, The Web of Whispers and The Lucky Trinket at 3 DP and minimum level 3. Records CHG-UAD-001 through CHG-UAD-006.

Universal Adept is complete at six cards. Universal Master is next. Book cards remain unchanged.
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/32_Adept_Abilities.xlsx
+++ b/review/abilities/workbooks/32_Adept_Abilities.xlsx
@@ -336,7 +336,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -783,7 +782,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The 91 shared Adept (level 3) abilities. The 30 class signatures are excluded here and reviewed in the ten class workbooks.</t>
+          <t>The 91 shared Adept (level 3) abilities plus the six Universal Adept abilities. The 30 class signatures are excluded here and reviewed in the ten class workbooks.</t>
         </is>
       </c>
     </row>
@@ -1120,8 +1119,8 @@
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="A19:D19"/>
@@ -1163,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V95"/>
+  <dimension ref="A1:V101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1200,7 +1199,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>91 shared cards. Signatures are excluded. Filter, decide, and add notes.</t>
+          <t>91 shared cards plus six Universal Adept cards. Signatures are excluded. Filter, decide, and add notes.</t>
         </is>
       </c>
     </row>
@@ -10912,6 +10911,685 @@
       <c r="V95" s="7" t="inlineStr">
         <is>
           <t>the-road-remembers.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>The Strong Arm</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>the-strong-arm</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Universal / Attack / Skill</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Main Action</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Brawn</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>One visible creature within 4 squares.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Instant.</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>One object per attack.</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Throw a two-handed weapon or improvised item at range 4; 3/4/6 physical damage.</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>You can throw weapons or improvised items that a normal person would require two hands to throw. Make a Brawn attack.
+• Weak: 3 physical damage.
+• Standard: 4 physical damage; the target is pushed 1 square.
+• Strong: 6 physical damage; the target is knocked Prone.</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>UA1; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>the-strong-arm.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>The Last Word</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>the-last-word</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Universal / Reaction / Recovery</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Self, when you enter Dying.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Instant.</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Once per scene; one Main Action.</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Take one Main Action when you enter Dying.</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>Take one Main Action before the Dying procedure. Then mark the wound and resolve Dying normally. Once per scene.</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>UA2; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>the-last-word.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>The Impossible Escape</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>the-impossible-escape</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Escape</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Maneuver</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Agility</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Self, when Grappled.</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Instant.</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>The squeeze is passive. The Grapple reduction is a Maneuver.</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Maneuver, Agility: 2/3/free Grapple reduction; squeeze through narrow gaps.</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Make an Agility check.
+• Weak: Reduce your Grappled rating by 2.
+• Standard: Reduce your Grappled rating by 3.
+• Strong: You are free of the Grapple; your Grappled rating becomes 0.
+You can squeeze through a gap wide enough for your head and shoulders at half Speed.</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>UA3; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>the-impossible-escape.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>A Name Worth Knowing</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>a-name-worth-knowing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Social</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Maneuver</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Self; the current location or situation.</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>The contact and favor persist until used or the fiction changes.</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Once per location or situation; one contact.</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Invent a contact and mutual favor; 2 Boons in social interactions with them.</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Invent one contact you know that may be here. You and the DA define the contact and the small favor they owe you or you owe them, such as a meal, a bed, an introduction, a rumor, a place to lie low, or a small loan. You have 2 Boons in your social interactions with them.</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>UA4; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>a-name-worth-knowing.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>The Web of Whispers</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>the-web-of-whispers</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Investigation / Passive</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Self; one question about a person, place, faction or event your network or research could plausibly know.</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>The answer and contact remain known.</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Once per scene; one question.</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Ask one question; the network answers truthfully from what it knows.</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Ask one question. The DA answers truthfully from what that network would know. The answer may be incomplete or point to a source. You also learn who can tell you more.</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>UA5; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>the-web-of-whispers.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>The Lucky Trinket</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>the-lucky-trinket</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Luck / Passive</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Self.</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>The trinket remains; the 2 Boons apply to one non-combat roll.</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Once a day; one non-combat roll.</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Once a day, a personal trinket grants 2 Boons on one non-combat roll.</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>You carry a personal trinket you believe is magical. It may or may not be. Once a day, when you make a non-combat roll, you can use the trinket to gain 2 Boons on that roll.</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>UA6; approved 2026-10-29. 2 Boons to the player confirmed.</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>the-lucky-trinket.md</t>
         </is>
       </c>
     </row>
@@ -11673,7 +12351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16685,6 +17363,318 @@
       <c r="K95" s="7" t="inlineStr">
         <is>
           <t>Single-discipline requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>The Strong Arm</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>the-strong-arm</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Main Action</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Attack</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>The Last Word</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>the-last-word</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Reaction</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>The Impossible Escape</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>the-impossible-escape</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Maneuver</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>A Name Worth Knowing</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>a-name-worth-knowing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Maneuver</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>The Web of Whispers</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>the-web-of-whispers</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>The Lucky Trinket</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>the-lucky-trinket</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Adept.</t>
         </is>
       </c>
     </row>
@@ -17624,118 +18614,502 @@
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UAD-001</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>the-strong-arm</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>The Strong Arm</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>the-strong-arm.md</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Main Action, Brawn, range 4; 3/4/6 physical damage; Standard push 1; Strong Prone; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA1 approved.</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O5" s="7" t="inlineStr"/>
-      <c r="P5" s="7" t="inlineStr"/>
-      <c r="Q5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>UA1; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="9" t="inlineStr"/>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UAD-002</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>the-last-word</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>The Last Word</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>the-last-word.md</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Reaction when entering Dying; take one Main Action before the Dying procedure; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA2 approved.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>UA2; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="7" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UAD-003</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>the-impossible-escape</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>The Impossible Escape</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>the-impossible-escape.md</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Maneuver, Agility; Grapple reduction 2/3/free; passive squeeze; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA3 approved.</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>UA3; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="9" t="inlineStr"/>
-      <c r="B8" s="9" t="inlineStr"/>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UAD-004</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>a-name-worth-knowing</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>A Name Worth Knowing</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>a-name-worth-knowing.md</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Maneuver, no roll; invent a contact and mutual favor; 2 Boons in social interactions with them; once per location or situation; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA4 approved.</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>UA4; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="7" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
-      <c r="N9" s="7" t="inlineStr"/>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UAD-005</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>the-web-of-whispers</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>The Web of Whispers</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>the-web-of-whispers.md</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Passive, no roll; ask one question and get a truthful answer from the network; once per scene; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA5 approved.</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>UA5; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="9" t="inlineStr"/>
-      <c r="B10" s="9" t="inlineStr"/>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="9" t="inlineStr"/>
-      <c r="M10" s="9" t="inlineStr"/>
-      <c r="N10" s="9" t="inlineStr"/>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UAD-006</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>UNI-03</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>the-lucky-trinket</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>The Lucky Trinket</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>the-lucky-trinket.md</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Passive; personal trinket; once a day, 2 Boons on one non-combat roll; 3 DP, Adept, minimum level 3.</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Universal Adept first pass; UA6 approved.</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
-      <c r="Q10" s="9" t="inlineStr"/>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>UA6; approved 2026-10-29. 2 Boons to the player confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="7" t="inlineStr"/>

</xml_diff>